<commit_message>
Fixed the solar eta
</commit_message>
<xml_diff>
--- a/AP1000_connection_results.xlsx
+++ b/AP1000_connection_results.xlsx
@@ -468,7 +468,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>943.5447572011866</v>
+        <v>949.7632182269745</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>543.9364592782728</v>
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>943.5447572011866</v>
+        <v>949.7632182024662</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>543.9364592782728</v>
@@ -496,7 +496,7 @@
         <v>5571000</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>2785600.000026754</v>
+        <v>2785600.000006875</v>
       </c>
     </row>
     <row r="4">
@@ -506,7 +506,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1887.089549560898</v>
+        <v>1899.526129216027</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>543.9364592782728</v>
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>1845.650911142159</v>
+        <v>1854.876678674435</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>543.9364592782728</v>
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>41.43851174611218</v>
+        <v>44.64957669618579</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>543.9364592782728</v>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>82.935</v>
+        <v>83.06999999999999</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>514.2650877161602</v>
@@ -582,16 +582,16 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>92.33941717575021</v>
+        <v>128.2111034820394</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>503.7892836524911</v>
+        <v>503.7293149982885</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>2830000</v>
+        <v>2826900</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>2677277.924528668</v>
+        <v>2677106.93180383</v>
       </c>
     </row>
     <row r="9">
@@ -601,146 +601,146 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>282.4959503506918</v>
+        <v>63.15758695117781</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>485.5272254246632</v>
+        <v>478.328610286492</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>2000000</v>
+        <v>1730600</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>2623871.180552623</v>
+        <v>2602164.910585302</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Inlet to moisture separator, outlet of HP turbine (exhaust)</t>
+          <t>Inlet to moisture separator, outlet of HP exhaust splitter</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>1387.880636668585</v>
+        <v>1424.203482658818</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>458.5268504151532</v>
+        <v>458.518972053546</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>1133000</v>
+        <v>1132800</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>2540015.126104773</v>
+        <v>2539966.681954201</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Inlet to MSR drain FWH (hot), outlet of moisture separator (liquid)</t>
+          <t>Inlet to MSR drain to deaerator valve, outlet of moisture separator (liquid)</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>168.1579025794896</v>
+        <v>172.5864322066738</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>458.5268504151532</v>
+        <v>458.518972053546</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>1133000</v>
+        <v>1132800</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>786861.3500349802</v>
+        <v>786826.3720510491</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Inlet to interstage heater 1 (cold), outlet of moisture separator (vapour)</t>
+          <t>Inlet to deaerator, outlet of MSR drain to deaerator valve</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>1219.722734563886</v>
+        <v>172.5864322066738</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>458.5268905386756</v>
+        <v>458.518972053546</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>1133000</v>
+        <v>1132800</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>2781714.860065929</v>
+        <v>786826.3720510491</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Inlet to interstage heater 2 (cold), outlet of interstage heater 1 (cold)</t>
+          <t>Inlet to interstage heater 1 (cold), outlet of moisture separator (vapour)</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>1219.722734563886</v>
+        <v>1251.617051527304</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>503.9770394251141</v>
+        <v>458.5190130708568</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>1110340</v>
+        <v>1132800</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>2895414.363083247</v>
+        <v>2781708.5397696</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Inlet to LP turbine stage 1, outlet of interstage heater 2 (cold)</t>
+          <t>Inlet to interstage heater 2 (cold), outlet of interstage heater 1 (cold)</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>1219.722734563886</v>
+        <v>1251.617051527304</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>527.7</v>
+        <v>502.7946156995406</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>1088133.2</v>
+        <v>1110144</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>2949983.851356694</v>
+        <v>2892691.060044494</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Inlet to interstage heater 2 drain valve, outlet of interstage heater 2 (hot)</t>
+          <t>Inlet to LP turbine stage 1, outlet of interstage heater 2 (cold)</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>41.43851174611218</v>
+        <v>1251.617051527304</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>541.9904787171338</v>
+        <v>527.7</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5403869.999999999</v>
+        <v>1087941.12</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>1179373.263663524</v>
+        <v>2949990.809897095</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Inlet to interstage heater drain merge, outlet of interstage heater 2 drain valve</t>
+          <t>Inlet to interstage heater 2 drain valve, outlet of interstage heater 2 (hot)</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>41.43851174611218</v>
+        <v>44.64957669618579</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>512.530576972507</v>
+        <v>541.9904787171338</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>3310634.25</v>
+        <v>5403869.999999999</v>
       </c>
       <c r="E16" s="4" t="n">
         <v>1179373.263663524</v>
@@ -749,11 +749,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Inlet to interstage heater drain merge, outlet of interstage heater 1 (hot)</t>
+          <t>Inlet to interstage heater drain merge, outlet of interstage heater 2 drain valve</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>82.935</v>
+        <v>44.64957669618579</v>
       </c>
       <c r="C17" s="2" t="n">
         <v>512.530576972507</v>
@@ -762,17 +762,17 @@
         <v>3310634.25</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>1034594.435890478</v>
+        <v>1179373.263663524</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Inlet to reheater drain FWH (hot), outlet of interstage heater drain merge</t>
+          <t>Inlet to interstage heater drain merge, outlet of interstage heater 1 (hot)</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>124.3735102451478</v>
+        <v>83.06999999999999</v>
       </c>
       <c r="C18" s="2" t="n">
         <v>512.530576972507</v>
@@ -781,824 +781,824 @@
         <v>3310634.25</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>1082831.551071167</v>
+        <v>1034594.435890478</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Inlet to reheater drain FWH drain valve, outlet of reheater drain FWH (hot)</t>
+          <t>Inlet to reheater drain FWH (hot), outlet of interstage heater drain merge</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>124.3735102451478</v>
+        <v>127.7195765246574</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>503.789283644132</v>
+        <v>512.530576972507</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>3211315.2225</v>
+        <v>3310634.25</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>993263.1508801192</v>
+        <v>1085207.768570942</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Inlet to HP FWH 2 shell merge, outlet of reheater drain FWH drain valve</t>
+          <t>Inlet to reheater drain FWH drain valve, outlet of reheater drain FWH (hot)</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>124.3735102451478</v>
+        <v>127.7195765246574</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>503.7892836524911</v>
+        <v>507.0633149616847</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>2830000</v>
+        <v>3211315.2225</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>993263.1508801192</v>
+        <v>1008660.451591974</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Inlet to HP FWH 2 (hot), outlet of HP FWH 2 shell merge</t>
+          <t>Inlet to HP FWH 2 shell merge, outlet of reheater drain FWH drain valve</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>216.7129274352899</v>
+        <v>127.7195765246574</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>503.7892836524911</v>
+        <v>503.7293149982885</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>2830000</v>
+        <v>2826900</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>1710806.606291927</v>
+        <v>1008660.451591974</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 3 shell merge, outlet of LP turbine stage 1 (stage 1 extraction)</t>
+          <t>Inlet to HP FWH 2 (hot), outlet of HP FWH 2 shell merge</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>104.148596195556</v>
+        <v>255.9306800142323</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>405.403119911276</v>
+        <v>503.7293149982885</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>289000</v>
+        <v>2826900</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>2715841.413721339</v>
+        <v>1844485.857596653</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Inlet to LP stage 1 exhaust splitter, outlet of LP turbine stage 1 (exhaust)</t>
+          <t>Inlet to LP FWH 4 (hot), outlet of LP turbine stage 1 (stage 1 extraction)</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>1115.574138259771</v>
+        <v>9.78623048777694</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>368.5938080797434</v>
+        <v>405.3914025973609</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>86000</v>
+        <v>288900</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>2538068.265773014</v>
+        <v>2715821.170307884</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 2 shell merge, outlet of LP stage 1 exhaust splitter</t>
+          <t>Inlet to LP FWH 3 shell merge, outlet of LP turbine stage 1 (stage 2 extraction)</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>15.38987548899179</v>
+        <v>79.71848685986375</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>368.5938080797434</v>
+        <v>401.4090908310928</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>86000</v>
+        <v>256500</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>2538068.265773014</v>
+        <v>2697195.181726462</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Inlet to LP turbine stage 2, outlet of LP stage 1 exhaust splitter</t>
+          <t>Inlet to LP stage 1 exhaust splitter, outlet of LP turbine stage 1 (exhaust)</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>1100.184262733621</v>
+        <v>1162.112333803341</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>368.5938080797434</v>
+        <v>368.7833302486509</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>86000</v>
+        <v>86600</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>2538068.265773014</v>
+        <v>2538855.421830092</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Inlet to LP stage 2 exhaust splitter, outlet of LP turbine stage 2</t>
+          <t>Inlet to LP FWH 2 shell merge, outlet of LP stage 1 exhaust splitter</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>1100.184262733621</v>
+        <v>43.79103138399749</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>349.3057275545186</v>
+        <v>368.7833302486509</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>40500</v>
+        <v>86600</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>2438466.382933303</v>
+        <v>2538855.421830092</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 1 shell merge, outlet of LP stage 2 exhaust splitter</t>
+          <t>Inlet to LP turbine stage 2, outlet of LP stage 1 exhaust splitter</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>89.21301716830783</v>
+        <v>1118.321302419344</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>349.3057275545186</v>
+        <v>368.7833302486509</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>40500</v>
+        <v>86600</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>2438466.382933303</v>
+        <v>2538855.421830092</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Inlet to LP turbine stage 3, outlet of LP stage 2 exhaust splitter</t>
+          <t>Inlet to LP stage 2 exhaust splitter, outlet of LP turbine stage 2</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>1010.971245591156</v>
+        <v>1118.321302419344</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>349.3057275545186</v>
+        <v>348.5830440496861</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>40500</v>
+        <v>39300</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>2438466.382933303</v>
+        <v>2434502.718127833</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Inlet to condenser merge, outlet of LP turbine stage 3</t>
+          <t>Inlet to LP FWH 1 shell merge, outlet of LP stage 2 exhaust splitter</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>1010.971245591156</v>
+        <v>69.94405904618078</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>312.1495642646744</v>
+        <v>348.5830440496861</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>7000</v>
+        <v>39300</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>2234112.301638001</v>
+        <v>2434502.718127833</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Inlet to main condenser (hot), outlet of condenser merge</t>
+          <t>Inlet to LP turbine stage 3, outlet of LP stage 2 exhaust splitter</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>1887.089515286098</v>
+        <v>1048.377243056483</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>312.1495642646744</v>
+        <v>348.5830440496861</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>7000</v>
+        <v>39300</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>1343502.043492448</v>
+        <v>2434502.718127833</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Inlet to condenser pump, outlet of main condenser (hot)</t>
+          <t>Inlet to condenser merge, outlet of LP turbine stage 3</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>1887.089515286098</v>
+        <v>1048.377243056483</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>312.1495629038336</v>
+        <v>315.7366090165625</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>7000</v>
+        <v>8466</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>163351.2627336636</v>
+        <v>2254348.054133357</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 1 (cold), outlet of condenser pump</t>
+          <t>Inlet to main condenser (hot), outlet of condenser merge</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>1887.089515286098</v>
+        <v>1251.617051600029</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>312.2536449070977</v>
+        <v>315.7366090165625</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>1200000</v>
+        <v>8466</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>164845.8466906142</v>
+        <v>1939074.705670959</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 2 (cold), outlet of LP FWH 1 (cold)</t>
+          <t>Inlet to condenser pump, outlet of main condenser (hot)</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>1887.089515286098</v>
+        <v>1251.617051600029</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>344.3057275581507</v>
+        <v>315.7366077216026</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>1164000</v>
+        <v>8466</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>298831.8490338236</v>
+        <v>178345.4598069412</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 3 (cold), outlet of LP FWH 2 (cold)</t>
+          <t>Inlet to LP FWH 1 (cold), outlet of condenser pump</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>1887.089515286098</v>
+        <v>1251.617051600029</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>363.5938081227878</v>
+        <v>315.8507351648028</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>1129080</v>
+        <v>1280000</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>379724.3095414915</v>
+        <v>179940.643566573</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 4 (cold), outlet of LP FWH 3 (cold)</t>
+          <t>Inlet to LP FWH 2 (cold), outlet of LP FWH 1 (cold)</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>1887.089515286098</v>
+        <v>1251.617051600029</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>400.4031199365085</v>
+        <v>346.3610438195695</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>1095207.6</v>
+        <v>1241600</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>535249.4284442024</v>
+        <v>307504.6420935374</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Inlet to MSR drain FWH (cold), outlet of LP FWH 4 (cold)</t>
+          <t>Inlet to LP FWH 3 (cold), outlet of LP FWH 2 (cold)</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>1887.089515286098</v>
+        <v>1251.617051600029</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>415.0484940683568</v>
+        <v>366.5613300555251</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>1062351.372</v>
+        <v>1204352</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>597746.5768960677</v>
+        <v>392259.7375220928</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Inlet to feed pump, outlet of MSR drain FWH (cold)</t>
+          <t>Inlet to LP FWH 4 (cold), outlet of LP FWH 3 (cold)</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>1887.089515286098</v>
+        <v>1251.617051600029</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>418.5360081394338</v>
+        <v>399.1870905498909</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>1030480.83084</v>
+        <v>1168221.44</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>612684.6597620897</v>
+        <v>530128.0337909439</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Inlet to HP FWH 1 (cold), outlet of feed pump</t>
+          <t>Inlet to LP FWH 4 to deaerator valve, outlet of LP FWH 4 (cold)</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>1887.089515286098</v>
+        <v>1251.617051600029</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>419.4125684340357</v>
+        <v>403.1693971712676</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>6292833.215261288</v>
+        <v>1133174.7968</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>619777.3609147848</v>
+        <v>547050.097548309</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Inlet to HP FWH 2 (cold), outlet of HP FWH 1 (cold)</t>
+          <t>Inlet to feed pump, outlet of deaerator</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>1887.089515286098</v>
+        <v>1899.526436502225</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>480.527225425323</v>
+        <v>458.518972053546</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>6104048.218803449</v>
+        <v>1132800</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>887255.445813226</v>
+        <v>786826.3373131653</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Inlet to reheater drain FWH (cold), outlet of HP FWH 2 (cold)</t>
+          <t>Inlet to HP FWH 1 (cold), outlet of feed pump</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>1887.089515286098</v>
+        <v>1899.526436502225</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>498.7892836530451</v>
+        <v>459.6011891174969</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>5920926.772239345</v>
+        <v>6292833.215261288</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>970561.5982088295</v>
+        <v>794098.4609609566</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Inlet to feedwater splitter, outlet of reheater drain FWH (cold)</t>
+          <t>Inlet to HP FWH 2 (cold), outlet of HP FWH 1 (cold)</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>1887.089515286098</v>
+        <v>1899.526436502225</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>500.073019711373</v>
+        <v>476.106610323407</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>5743298.969072165</v>
+        <v>6104048.218803449</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>976464.8350410637</v>
+        <v>867376.6962175592</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Inlet to steam generator 1, outlet of feedwater splitter</t>
+          <t>Inlet to reheater drain FWH (cold), outlet of HP FWH 2 (cold)</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>943.5447572011866</v>
+        <v>1899.526436502225</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>500.073019711373</v>
+        <v>501.5073149689487</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>5743298.969072165</v>
+        <v>5920926.772239345</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>976464.8350410637</v>
+        <v>983163.0741318994</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Inlet to steam generator 2, outlet of feedwater splitter</t>
+          <t>Inlet to feedwater splitter, outlet of reheater drain FWH (cold)</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>943.5447572011866</v>
+        <v>1899.526436502225</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>500.073019711373</v>
+        <v>502.6221224510821</v>
       </c>
       <c r="D43" s="3" t="n">
         <v>5743298.969072165</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>976464.8350410637</v>
+        <v>988309.9309563471</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Inlet to HP FWH merge, outlet of HP FWH drain valve 2</t>
+          <t>Inlet to steam generator 1, outlet of feedwater splitter</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>216.7129274352899</v>
+        <v>949.7632182269745</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>485.5272254246632</v>
+        <v>502.6221224510821</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>2000000</v>
+        <v>5743298.969072165</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>985394.5667971369</v>
+        <v>988309.9309563471</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Inlet to HP FWH 1 (hot), outlet of HP FWH merge</t>
+          <t>Inlet to steam generator 2, outlet of feedwater splitter</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>499.2088786699381</v>
+        <v>949.7632182024662</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>485.5272254246632</v>
+        <v>502.6221224510821</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>2000000</v>
+        <v>5743298.969072165</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>1912587.628834541</v>
+        <v>988309.9309563471</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Inlet to HP FWH drain valve 1, outlet of HP FWH 1 (hot)</t>
+          <t>Inlet to HP FWH merge, outlet of HP FWH drain valve 2</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>499.2088786699381</v>
+        <v>255.9306800142323</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>483.9922741299346</v>
+        <v>478.328610286492</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>1940000</v>
+        <v>1730600</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>901477.6268916579</v>
+        <v>985115.3214277856</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Inlet to HP FWH drain valve 2, outlet of HP FWH 2 (hot)</t>
+          <t>Inlet to HP FWH 1 (hot), outlet of HP FWH merge</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>216.7129274352899</v>
+        <v>319.0882679059834</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>502.1283059039064</v>
+        <v>478.328610286492</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>2745100</v>
+        <v>1730600</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>985394.5667971369</v>
+        <v>1305180.211278818</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 4 (hot), outlet of HP FWH drain valve 1</t>
+          <t>Inlet to HP FWH drain valve 1, outlet of HP FWH 1 (hot)</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>499.2088786699381</v>
+        <v>319.0882679059834</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>431.9764772652176</v>
+        <v>476.842455091916</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>600000</v>
+        <v>1678682</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>901477.6268916579</v>
+        <v>868956.2503961392</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 4 drain valve, outlet of LP FWH 4 (hot)</t>
+          <t>Inlet to HP FWH drain valve 2, outlet of HP FWH 2 (hot)</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>499.2088786699381</v>
+        <v>255.9306800142323</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>430.7898350799921</v>
+        <v>502.0687558277129</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>582000</v>
+        <v>2742093</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>665228.3957644919</v>
+        <v>985115.3214277856</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 3 shell merge, outlet of LP FWH 4 drain valve</t>
+          <t>Inlet to deaerator, outlet of HP FWH drain valve 1</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>499.2088786699381</v>
+        <v>319.0882679059834</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>405.403119911276</v>
+        <v>458.518972053546</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>289000</v>
+        <v>1132800</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>665228.3957644919</v>
+        <v>868956.2503961392</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 3 (hot), outlet of LP FWH 3 shell merge</t>
+          <t>Inlet to LP FWH 4 drain valve, outlet of LP FWH 4 (hot)</t>
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>771.5153775343325</v>
+        <v>9.78623048777694</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>405.403119911276</v>
+        <v>404.3631444051296</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>289000</v>
+        <v>280232.9999999999</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>932018.2958258714</v>
+        <v>551561.5936657074</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 3 drain valve, outlet of LP FWH 3 (hot)</t>
+          <t>Inlet to LP FWH 3 shell merge, outlet of LP FWH 4 drain valve</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>771.5153775343325</v>
+        <v>9.78623048777694</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>404.3747943041712</v>
+        <v>401.4090908310928</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>280330</v>
+        <v>256500</v>
       </c>
       <c r="E52" s="4" t="n">
-        <v>551611.3328940334</v>
+        <v>551561.5936657074</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 2 shell merge, outlet of LP FWH 3 drain valve</t>
+          <t>Inlet to LP FWH 3 (hot), outlet of LP FWH 3 shell merge</t>
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>771.5153775343325</v>
+        <v>89.50471734764068</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>368.5938080797434</v>
+        <v>401.4090908310928</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>86000</v>
+        <v>256500</v>
       </c>
       <c r="E53" s="4" t="n">
-        <v>551611.3328940334</v>
+        <v>2462596.759257218</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 2 (hot), outlet of LP FWH 2 shell merge</t>
+          <t>Inlet to LP FWH 3 drain valve, outlet of LP FWH 3 (hot)</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>786.9052525339273</v>
+        <v>89.50471734764068</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>368.5938080797434</v>
+        <v>400.4036179890857</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>86000</v>
+        <v>248805</v>
       </c>
       <c r="E54" s="4" t="n">
-        <v>590461.4035559439</v>
+        <v>534672.5636695368</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 2 drain valve, outlet of LP FWH 2 (hot)</t>
+          <t>Inlet to LP FWH 2 shell merge, outlet of LP FWH 3 drain valve</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>786.9052525339273</v>
+        <v>89.50471734764068</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>367.7661293271289</v>
+        <v>368.7833302486509</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>83420</v>
+        <v>86600</v>
       </c>
       <c r="E55" s="4" t="n">
-        <v>396471.9572653652</v>
+        <v>534672.5636695368</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 1 shell merge, outlet of LP FWH 2 drain valve</t>
+          <t>Inlet to LP FWH 2 (hot), outlet of LP FWH 2 shell merge</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>786.9052525339273</v>
+        <v>133.2957542778902</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>349.3057275545186</v>
+        <v>368.7833302486509</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>40500</v>
+        <v>86600</v>
       </c>
       <c r="E56" s="4" t="n">
-        <v>396471.9572653652</v>
+        <v>1193097.386605988</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 1 (hot), outlet of LP FWH 1 shell merge</t>
+          <t>Inlet to LP FWH 2 drain valve, outlet of LP FWH 2 (hot)</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>876.1182692310272</v>
+        <v>133.2957542778902</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>349.3057275545186</v>
+        <v>367.9546772634875</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>40500</v>
+        <v>84002</v>
       </c>
       <c r="E57" s="4" t="n">
-        <v>604403.3405785144</v>
+        <v>397266.171149075</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 1 drain valve, outlet of LP FWH 1 (hot)</t>
+          <t>Inlet to LP FWH 1 shell merge, outlet of LP FWH 2 drain valve</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>876.1182692310272</v>
+        <v>133.2957542778902</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>348.5738935596557</v>
+        <v>348.5830440496861</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>39285</v>
+        <v>39300</v>
       </c>
       <c r="E58" s="4" t="n">
-        <v>315808.079924843</v>
+        <v>397266.171149075</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Inlet to condenser merge, outlet of LP FWH 1 drain valve</t>
+          <t>Inlet to LP FWH 1 (hot), outlet of LP FWH 1 shell merge</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>876.1182692310272</v>
+        <v>203.2398135549068</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>312.1495642646744</v>
+        <v>348.5830440496861</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>7000</v>
+        <v>39300</v>
       </c>
       <c r="E59" s="4" t="n">
-        <v>315808.079924843</v>
+        <v>1098371.883194878</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Inlet to MSR drain FWH drain valve, outlet of MSR drain FWH (hot)</t>
+          <t>Inlet to LP FWH 1 drain valve, outlet of LP FWH 1 (hot)</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>168.1579025794896</v>
+        <v>203.2398135549068</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>420.0484940829248</v>
+        <v>347.8546727538545</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>1099010</v>
+        <v>38121</v>
       </c>
       <c r="E60" s="4" t="n">
-        <v>619224.2706995687</v>
+        <v>312791.1722464436</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 3 shell merge, outlet of MSR drain FWH drain valve</t>
+          <t>Inlet to condenser merge, outlet of LP FWH 1 drain valve</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>168.1579025794896</v>
+        <v>203.2398135549068</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>405.403119911276</v>
+        <v>315.7366090165625</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>289000</v>
+        <v>8466</v>
       </c>
       <c r="E61" s="4" t="n">
-        <v>619224.2706995687</v>
+        <v>312791.1722464436</v>
       </c>
     </row>
     <row r="62">
@@ -1608,7 +1608,7 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>44361.55513331488</v>
+        <v>43897.60316817585</v>
       </c>
       <c r="C62" s="2" t="n">
         <v>288.15</v>
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>44361.55513331488</v>
+        <v>43897.60316817585</v>
       </c>
       <c r="C63" s="2" t="n">
         <v>300.15</v>

</xml_diff>

<commit_message>
Came up with an intersting 2D test for config 2
</commit_message>
<xml_diff>
--- a/AP1000_connection_results.xlsx
+++ b/AP1000_connection_results.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Connections" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Connections'!$A$1:$E$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Connections'!$A$1:$E$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="88" customWidth="1" min="1" max="1"/>
@@ -468,7 +468,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>949.7632182269745</v>
+        <v>953.2513493266538</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>543.9364592782728</v>
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>949.7632182024662</v>
+        <v>953.2513493076403</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>543.9364592782728</v>
@@ -496,7 +496,7 @@
         <v>5571000</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>2785600.000006875</v>
+        <v>2785600.000005253</v>
       </c>
     </row>
     <row r="4">
@@ -506,7 +506,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1899.526129216027</v>
+        <v>1906.502416208381</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>543.9364592782728</v>
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>1854.876678674435</v>
+        <v>1855.280542954665</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>543.9364592782728</v>
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>44.64957669618579</v>
+        <v>51.22197468759215</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>543.9364592782728</v>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>83.06999999999999</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>514.2650877161602</v>
@@ -572,7 +572,7 @@
         <v>3413025</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>2706769.891396322</v>
+        <v>2707942.955850471</v>
       </c>
     </row>
     <row r="8">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>128.2111034820394</v>
+        <v>120.9311164912711</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>503.7293149982885</v>
@@ -591,7 +591,7 @@
         <v>2826900</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>2677106.93180383</v>
+        <v>2675340.970985502</v>
       </c>
     </row>
     <row r="9">
@@ -601,16 +601,16 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>63.15758695117781</v>
+        <v>72.45505544482978</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>478.328610286492</v>
+        <v>479.869559856783</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>1730600</v>
+        <v>1785742.14</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>2602164.910585302</v>
+        <v>2600643.094588067</v>
       </c>
     </row>
     <row r="10">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>1424.203482658818</v>
+        <v>1424.504054221518</v>
       </c>
       <c r="C10" s="2" t="n">
         <v>458.518972053546</v>
@@ -629,7 +629,7 @@
         <v>1132800</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>2539966.681954201</v>
+        <v>2530551.428779312</v>
       </c>
     </row>
     <row r="11">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>172.5864322066738</v>
+        <v>179.3460930836507</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>458.518972053546</v>
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>172.5864322066738</v>
+        <v>179.3460930836507</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>458.518972053546</v>
@@ -677,7 +677,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>1251.617051527304</v>
+        <v>1245.157962213027</v>
       </c>
       <c r="C13" s="2" t="n">
         <v>458.5190130708568</v>
@@ -696,26 +696,26 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>1251.617051527304</v>
+        <v>1245.157962213027</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>502.7946156995406</v>
+        <v>500.4387233820347</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>1110144</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>2892691.060044494</v>
+        <v>2887229.6963241</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Inlet to LP turbine stage 1, outlet of interstage heater 2 (cold)</t>
+          <t>Inlet to LP turbine inlet splitter, outlet of interstage heater 2 (cold)</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>1251.617051527304</v>
+        <v>1245.157962213027</v>
       </c>
       <c r="C15" s="2" t="n">
         <v>527.7</v>
@@ -730,258 +730,258 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Inlet to interstage heater 2 drain valve, outlet of interstage heater 2 (hot)</t>
+          <t>Inlet to LP turbine 1, outlet of LP turbine inlet splitter</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>44.64957669618579</v>
+        <v>9.750833827809432</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>541.9904787171338</v>
+        <v>527.7000000001055</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>5403869.999999999</v>
+        <v>1087941.12</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>1179373.263663524</v>
+        <v>2949990.809897095</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Inlet to interstage heater drain merge, outlet of interstage heater 2 drain valve</t>
+          <t>Inlet to LP turbine 2, outlet of LP turbine inlet splitter</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>44.64957669618579</v>
+        <v>123.4308372206955</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>512.530576972507</v>
+        <v>527.7000000001055</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>3310634.25</v>
+        <v>1087941.12</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>1179373.263663524</v>
+        <v>2949990.809897095</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Inlet to interstage heater drain merge, outlet of interstage heater 1 (hot)</t>
+          <t>Inlet to LP turbine 3, outlet of LP turbine inlet splitter</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>83.06999999999999</v>
+        <v>1111.97629117311</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>512.530576972507</v>
+        <v>527.7000000001055</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>3310634.25</v>
+        <v>1087941.12</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>1034594.435890478</v>
+        <v>2949990.809897095</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Inlet to reheater drain FWH (hot), outlet of interstage heater drain merge</t>
+          <t>Inlet to interstage heater 2 drain valve, outlet of interstage heater 2 (hot)</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>127.7195765246574</v>
+        <v>51.22197468759215</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>512.530576972507</v>
+        <v>541.9904787171338</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>3310634.25</v>
+        <v>5403869.999999999</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>1085207.768570942</v>
+        <v>1259936.442318106</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Inlet to reheater drain FWH drain valve, outlet of reheater drain FWH (hot)</t>
+          <t>Inlet to interstage heater drain merge, outlet of interstage heater 2 drain valve</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>127.7195765246574</v>
+        <v>51.22197468759215</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>507.0633149616847</v>
+        <v>512.530576972507</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>3211315.2225</v>
+        <v>3310634.25</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>1008660.451591974</v>
+        <v>1259936.442318106</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Inlet to HP FWH 2 shell merge, outlet of reheater drain FWH drain valve</t>
+          <t>Inlet to interstage heater drain merge, outlet of interstage heater 1 (hot)</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>127.7195765246574</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>503.7293149982885</v>
+        <v>512.530576972507</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>2826900</v>
+        <v>3310634.25</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>1008660.451591974</v>
+        <v>1123015.229741286</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Inlet to HP FWH 2 (hot), outlet of HP FWH 2 shell merge</t>
+          <t>Inlet to reheater drain FWH (hot), outlet of interstage heater drain merge</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>255.9306800142323</v>
+        <v>134.1219744994448</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>503.7293149982885</v>
+        <v>512.530576972507</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>2826900</v>
+        <v>3310634.25</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>1844485.857596653</v>
+        <v>1175306.249473965</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 4 (hot), outlet of LP turbine stage 1 (stage 1 extraction)</t>
+          <t>Inlet to reheater drain FWH drain valve, outlet of reheater drain FWH (hot)</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>9.78623048777694</v>
+        <v>134.1219744994448</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>405.3914025973609</v>
+        <v>507.063314963205</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>288900</v>
+        <v>3211315.2225</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>2715821.170307884</v>
+        <v>1008660.451595714</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 3 shell merge, outlet of LP turbine stage 1 (stage 2 extraction)</t>
+          <t>Inlet to HP FWH 2 shell merge, outlet of reheater drain FWH drain valve</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>79.71848685986375</v>
+        <v>134.1219744994448</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>401.4090908310928</v>
+        <v>503.7293149982885</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>256500</v>
+        <v>2826900</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>2697195.181726462</v>
+        <v>1008660.451595714</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Inlet to LP stage 1 exhaust splitter, outlet of LP turbine stage 1 (exhaust)</t>
+          <t>Inlet to HP FWH 2 (hot), outlet of HP FWH 2 shell merge</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>1162.112333803341</v>
+        <v>255.0530909258279</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>368.7833302486509</v>
+        <v>503.7293149982885</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>86600</v>
+        <v>2826900</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>2538855.421830092</v>
+        <v>1798901.94704922</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 2 shell merge, outlet of LP stage 1 exhaust splitter</t>
+          <t>Inlet to LP FWH 4 (hot), outlet of LP turbine 1</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>43.79103138399749</v>
+        <v>9.750833827809432</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>368.7833302486509</v>
+        <v>405.3914025973609</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>86600</v>
+        <v>288900</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>2538855.421830092</v>
+        <v>2712468.230401031</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Inlet to LP turbine stage 2, outlet of LP stage 1 exhaust splitter</t>
+          <t>Inlet to LP FWH 3 shell merge, outlet of LP turbine 2 (stage 1 extraction)</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>1118.321302419344</v>
+        <v>79.63812614213074</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>368.7833302486509</v>
+        <v>401.4090908310928</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>86600</v>
+        <v>256500</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>2538855.421830092</v>
+        <v>2688202.957196377</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Inlet to LP stage 2 exhaust splitter, outlet of LP turbine stage 2</t>
+          <t>Inlet to LP FWH 2 shell merge, outlet of LP turbine 2 (exhaust)</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>1118.321302419344</v>
+        <v>43.79271107780325</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>348.5830440496861</v>
+        <v>368.7833302486509</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>39300</v>
+        <v>86600</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>2434502.718127833</v>
+        <v>2526635.759006064</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 1 shell merge, outlet of LP stage 2 exhaust splitter</t>
+          <t>Inlet to LP FWH 1 shell merge, outlet of LP turbine 3 (stage 1 extraction)</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>69.94405904618078</v>
+        <v>68.46701444654232</v>
       </c>
       <c r="C29" s="2" t="n">
         <v>348.5830440496861</v>
@@ -990,36 +990,36 @@
         <v>39300</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>2434502.718127833</v>
+        <v>2468236.054069106</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Inlet to LP turbine stage 3, outlet of LP stage 2 exhaust splitter</t>
+          <t>Inlet to condenser merge, outlet of LP turbine 3 (exhaust)</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>1048.377243056483</v>
+        <v>1043.509276393351</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>348.5830440496861</v>
+        <v>315.7366090165625</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>39300</v>
+        <v>8466</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>2434502.718127833</v>
+        <v>2295406.299437628</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Inlet to condenser merge, outlet of LP turbine stage 3</t>
+          <t>Inlet to main condenser (hot), outlet of condenser merge</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>1048.377243056483</v>
+        <v>1245.157962290019</v>
       </c>
       <c r="C31" s="2" t="n">
         <v>315.7366090165625</v>
@@ -1028,384 +1028,384 @@
         <v>8466</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>2254348.054133357</v>
+        <v>1974329.291941202</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Inlet to main condenser (hot), outlet of condenser merge</t>
+          <t>Inlet to condenser pump, outlet of main condenser (hot)</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>1251.617051600029</v>
+        <v>1245.157962290019</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>315.7366090165625</v>
+        <v>315.7366077216026</v>
       </c>
       <c r="D32" s="3" t="n">
         <v>8466</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>1939074.705670959</v>
+        <v>178345.4598069412</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Inlet to condenser pump, outlet of main condenser (hot)</t>
+          <t>Inlet to LP FWH 1 (cold), outlet of condenser pump</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>1251.617051600029</v>
+        <v>1245.157962290019</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>315.7366077216026</v>
+        <v>315.8526446808814</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>8466</v>
+        <v>1280000</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>178345.4598069412</v>
+        <v>179948.6194417125</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 1 (cold), outlet of condenser pump</t>
+          <t>Inlet to LP FWH 2 (cold), outlet of LP FWH 1 (cold)</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>1251.617051600029</v>
+        <v>1245.157962290019</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>315.8507351648028</v>
+        <v>346.3610438195695</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>1280000</v>
+        <v>1241600</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>179940.643566573</v>
+        <v>307504.6420935374</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 2 (cold), outlet of LP FWH 1 (cold)</t>
+          <t>Inlet to LP FWH 3 (cold), outlet of LP FWH 2 (cold)</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>1251.617051600029</v>
+        <v>1245.157962290019</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>346.3610438195695</v>
+        <v>366.5613300555251</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>1241600</v>
+        <v>1204352</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>307504.6420935374</v>
+        <v>392259.7375220928</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 3 (cold), outlet of LP FWH 2 (cold)</t>
+          <t>Inlet to LP FWH 4 (cold), outlet of LP FWH 3 (cold)</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>1251.617051600029</v>
+        <v>1245.157962290019</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>366.5613300555251</v>
+        <v>399.1870905498909</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>1204352</v>
+        <v>1168221.44</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>392259.7375220928</v>
+        <v>530128.0337909439</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 4 (cold), outlet of LP FWH 3 (cold)</t>
+          <t>Inlet to LP FWH 4 to deaerator valve, outlet of LP FWH 4 (cold)</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>1251.617051600029</v>
+        <v>1245.157962290019</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>399.1870905498909</v>
+        <v>403.1693971712676</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>1168221.44</v>
+        <v>1133174.7968</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>530128.0337909439</v>
+        <v>547050.097548309</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 4 to deaerator valve, outlet of LP FWH 4 (cold)</t>
+          <t>Inlet to feed pump, outlet of deaerator</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>1251.617051600029</v>
+        <v>1906.502698674531</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>403.1693971712676</v>
+        <v>458.518972053546</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>1133174.7968</v>
+        <v>1132800</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>547050.097548309</v>
+        <v>786826.3373131653</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Inlet to feed pump, outlet of deaerator</t>
+          <t>Inlet to HP FWH 1 (cold), outlet of feed pump</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>1899.526436502225</v>
+        <v>1906.502698674531</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>458.518972053546</v>
+        <v>459.6094388690083</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>1132800</v>
+        <v>6292833.215261288</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>786826.3373131653</v>
+        <v>794134.8209930366</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Inlet to HP FWH 1 (cold), outlet of feed pump</t>
+          <t>Inlet to HP FWH 2 (cold), outlet of HP FWH 1 (cold)</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>1899.526436502225</v>
+        <v>1906.502698674531</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>459.6011891174969</v>
+        <v>477.6475598856132</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>6292833.215261288</v>
+        <v>6104048.218803449</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>794098.4609609566</v>
+        <v>874294.2042124182</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Inlet to HP FWH 2 (cold), outlet of HP FWH 1 (cold)</t>
+          <t>Inlet to reheater drain FWH (cold), outlet of HP FWH 2 (cold)</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>1899.526436502225</v>
+        <v>1906.502698674531</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>476.106610323407</v>
+        <v>501.5073149665665</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>6104048.218803449</v>
+        <v>5920926.772239345</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>867376.6962175592</v>
+        <v>983163.0741208255</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Inlet to reheater drain FWH (cold), outlet of HP FWH 2 (cold)</t>
+          <t>Inlet to feedwater splitter, outlet of reheater drain FWH (cold)</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>1899.526436502225</v>
+        <v>1906.502698674531</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>501.5073149689487</v>
+        <v>504.0328009686768</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>5920926.772239345</v>
+        <v>5743298.969072165</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>983163.0741318994</v>
+        <v>994886.5630314471</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Inlet to feedwater splitter, outlet of reheater drain FWH (cold)</t>
+          <t>Inlet to steam generator 1, outlet of feedwater splitter</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>1899.526436502225</v>
+        <v>953.2513493266538</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>502.6221224510821</v>
+        <v>504.0328009686768</v>
       </c>
       <c r="D43" s="3" t="n">
         <v>5743298.969072165</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>988309.9309563471</v>
+        <v>994886.5630314471</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Inlet to steam generator 1, outlet of feedwater splitter</t>
+          <t>Inlet to steam generator 2, outlet of feedwater splitter</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>949.7632182269745</v>
+        <v>953.2513493076403</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>502.6221224510821</v>
+        <v>504.0328009686768</v>
       </c>
       <c r="D44" s="3" t="n">
         <v>5743298.969072165</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>988309.9309563471</v>
+        <v>994886.5630314471</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Inlet to steam generator 2, outlet of feedwater splitter</t>
+          <t>Inlet to HP FWH merge, outlet of HP FWH drain valve 2</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>949.7632182024662</v>
+        <v>255.0530909258279</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>502.6221224510821</v>
+        <v>479.869559856783</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>5743298.969072165</v>
+        <v>1785742.14</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>988309.9309563471</v>
+        <v>985115.3214277856</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Inlet to HP FWH merge, outlet of HP FWH drain valve 2</t>
+          <t>Inlet to HP FWH 1 (hot), outlet of HP FWH merge</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>255.9306800142323</v>
+        <v>327.5081472475683</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>478.328610286492</v>
+        <v>479.869559856783</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>1730600</v>
+        <v>1785742.14</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>985115.3214277856</v>
+        <v>1342520.645961444</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Inlet to HP FWH 1 (hot), outlet of HP FWH merge</t>
+          <t>Inlet to HP FWH drain valve 1, outlet of HP FWH 1 (hot)</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>319.0882679059834</v>
+        <v>327.5081472475683</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>478.328610286492</v>
+        <v>478.3730048178063</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>1730600</v>
+        <v>1732169.8758</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>1305180.211278818</v>
+        <v>875893.8318121601</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Inlet to HP FWH drain valve 1, outlet of HP FWH 1 (hot)</t>
+          <t>Inlet to HP FWH drain valve 2, outlet of HP FWH 2 (hot)</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>319.0882679059834</v>
+        <v>255.0530909258279</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>476.842455091916</v>
+        <v>502.0687558277129</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>1678682</v>
+        <v>2742093</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>868956.2503961392</v>
+        <v>985115.3214277856</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Inlet to HP FWH drain valve 2, outlet of HP FWH 2 (hot)</t>
+          <t>Inlet to deaerator, outlet of HP FWH drain valve 1</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>255.9306800142323</v>
+        <v>327.5081472475683</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>502.0687558277129</v>
+        <v>458.518972053546</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>2742093</v>
+        <v>1132800</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>985115.3214277856</v>
+        <v>875893.8318121601</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Inlet to deaerator, outlet of HP FWH drain valve 1</t>
+          <t>Inlet to LP FWH 4 drain valve, outlet of LP FWH 4 (hot)</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>319.0882679059834</v>
+        <v>9.750833827809432</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>458.518972053546</v>
+        <v>404.3631444051296</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>1132800</v>
+        <v>280232.9999999999</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>868956.2503961392</v>
+        <v>551561.5936657074</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 4 drain valve, outlet of LP FWH 4 (hot)</t>
+          <t>Inlet to LP FWH 3 shell merge, outlet of LP FWH 4 drain valve</t>
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>9.78623048777694</v>
+        <v>9.750833827809432</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>404.3631444051296</v>
+        <v>401.4090908310928</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>280232.9999999999</v>
+        <v>256500</v>
       </c>
       <c r="E51" s="4" t="n">
         <v>551561.5936657074</v>
@@ -1414,11 +1414,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 3 shell merge, outlet of LP FWH 4 drain valve</t>
+          <t>Inlet to LP FWH 3 (hot), outlet of LP FWH 3 shell merge</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>9.78623048777694</v>
+        <v>89.38895997070163</v>
       </c>
       <c r="C52" s="2" t="n">
         <v>401.4090908310928</v>
@@ -1427,42 +1427,42 @@
         <v>256500</v>
       </c>
       <c r="E52" s="4" t="n">
-        <v>551561.5936657074</v>
+        <v>2455131.268088248</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 3 (hot), outlet of LP FWH 3 shell merge</t>
+          <t>Inlet to LP FWH 3 drain valve, outlet of LP FWH 3 (hot)</t>
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>89.50471734764068</v>
+        <v>89.38895997070163</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>401.4090908310928</v>
+        <v>400.4036179890857</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>256500</v>
+        <v>248805</v>
       </c>
       <c r="E53" s="4" t="n">
-        <v>2462596.759257218</v>
+        <v>534672.5636695368</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 3 drain valve, outlet of LP FWH 3 (hot)</t>
+          <t>Inlet to LP FWH 2 shell merge, outlet of LP FWH 3 drain valve</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>89.50471734764068</v>
+        <v>89.38895997070163</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>400.4036179890857</v>
+        <v>368.7833302486509</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>248805</v>
+        <v>86600</v>
       </c>
       <c r="E54" s="4" t="n">
         <v>534672.5636695368</v>
@@ -1471,11 +1471,11 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 2 shell merge, outlet of LP FWH 3 drain valve</t>
+          <t>Inlet to LP FWH 2 (hot), outlet of LP FWH 2 shell merge</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>89.50471734764068</v>
+        <v>133.1816767515784</v>
       </c>
       <c r="C55" s="2" t="n">
         <v>368.7833302486509</v>
@@ -1484,42 +1484,42 @@
         <v>86600</v>
       </c>
       <c r="E55" s="4" t="n">
-        <v>534672.5636695368</v>
+        <v>1189668.579565586</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 2 (hot), outlet of LP FWH 2 shell merge</t>
+          <t>Inlet to LP FWH 2 drain valve, outlet of LP FWH 2 (hot)</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>133.2957542778902</v>
+        <v>133.1816767515784</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>368.7833302486509</v>
+        <v>367.9546772634875</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>86600</v>
+        <v>84002</v>
       </c>
       <c r="E56" s="4" t="n">
-        <v>1193097.386605988</v>
+        <v>397266.171149075</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 2 drain valve, outlet of LP FWH 2 (hot)</t>
+          <t>Inlet to LP FWH 1 shell merge, outlet of LP FWH 2 drain valve</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>133.2957542778902</v>
+        <v>133.1816767515784</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>367.9546772634875</v>
+        <v>348.5830440496861</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>84002</v>
+        <v>39300</v>
       </c>
       <c r="E57" s="4" t="n">
         <v>397266.171149075</v>
@@ -1528,11 +1528,11 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 1 shell merge, outlet of LP FWH 2 drain valve</t>
+          <t>Inlet to LP FWH 1 (hot), outlet of LP FWH 1 shell merge</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>133.2957542778902</v>
+        <v>201.6486914288401</v>
       </c>
       <c r="C58" s="2" t="n">
         <v>348.5830440496861</v>
@@ -1541,42 +1541,42 @@
         <v>39300</v>
       </c>
       <c r="E58" s="4" t="n">
-        <v>397266.171149075</v>
+        <v>1100435.255690556</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 1 (hot), outlet of LP FWH 1 shell merge</t>
+          <t>Inlet to LP FWH 1 drain valve, outlet of LP FWH 1 (hot)</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>203.2398135549068</v>
+        <v>201.6486914288401</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>348.5830440496861</v>
+        <v>347.8546727538545</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>39300</v>
+        <v>38121</v>
       </c>
       <c r="E59" s="4" t="n">
-        <v>1098371.883194878</v>
+        <v>312791.1722464436</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Inlet to LP FWH 1 drain valve, outlet of LP FWH 1 (hot)</t>
+          <t>Inlet to condenser merge, outlet of LP FWH 1 drain valve</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>203.2398135549068</v>
+        <v>201.6486914288401</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>347.8546727538545</v>
+        <v>315.7366090165625</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>38121</v>
+        <v>8466</v>
       </c>
       <c r="E60" s="4" t="n">
         <v>312791.1722464436</v>
@@ -1585,62 +1585,43 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Inlet to condenser merge, outlet of LP FWH 1 drain valve</t>
+          <t>Inlet to main condenser (cold), outlet of cooling water source</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>203.2398135549068</v>
+        <v>152899.3619716934</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>315.7366090165625</v>
+        <v>303.65</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>8466</v>
+        <v>120000</v>
       </c>
       <c r="E61" s="4" t="n">
-        <v>312791.1722464436</v>
+        <v>127929.4036756703</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Inlet to main condenser (cold), outlet of cooling water source</t>
+          <t>Inlet to cooling water sink, outlet of main condenser (cold)</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>43897.60316817585</v>
+        <v>152899.3619716934</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>288.15</v>
+        <v>307.15</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>120000</v>
+        <v>117600</v>
       </c>
       <c r="E62" s="4" t="n">
-        <v>63094.70995793411</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Inlet to cooling water sink, outlet of main condenser (cold)</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="n">
-        <v>43897.60316817585</v>
-      </c>
-      <c r="C63" s="2" t="n">
-        <v>300.15</v>
-      </c>
-      <c r="D63" s="3" t="n">
-        <v>117600</v>
-      </c>
-      <c r="E63" s="4" t="n">
-        <v>113296.9692625922</v>
+        <v>142555.25720918</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E63"/>
+  <autoFilter ref="A1:E62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>